<commit_message>
Improve UI/UX across receipt form, tables, and settings - add date picker, Lei currency, grand total, edit/save workflow, consistent styling
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/templates/Template-deviz.xlsx
+++ b/templates/Template-deviz.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{76E170DE-EFC2-4ED5-982D-809527E1A88F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BA8E0562-E983-4298-B840-BAC4B79381D4}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{76E170DE-EFC2-4ED5-982D-809527E1A88F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A94D8376-4675-402E-BC05-87479C6FB00F}"/>
   <bookViews>
-    <workbookView xWindow="-28020" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="54">
   <si>
     <t xml:space="preserve">S.C. NELOAICA S.R.L.           DEVIZ DE REPARATIE </t>
   </si>
@@ -115,9 +115,6 @@
   </si>
   <si>
     <t>H</t>
-  </si>
-  <si>
-    <t>CONSTATARE-DIAGNOZA</t>
   </si>
   <si>
     <t>Total manopera</t>
@@ -1227,6 +1224,10 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1583,11 +1584,11 @@
       </c>
       <c r="B10" s="12"/>
       <c r="C10" s="13" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D10" s="14"/>
       <c r="E10" s="14" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F10" s="107"/>
     </row>
@@ -1848,9 +1849,7 @@
     </row>
     <row r="36" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="59"/>
-      <c r="B36" s="60" t="s">
-        <v>28</v>
-      </c>
+      <c r="B36" s="60"/>
       <c r="C36" s="61"/>
       <c r="D36" s="62"/>
       <c r="E36" s="63"/>
@@ -1862,7 +1861,7 @@
     <row r="37" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="65"/>
       <c r="B37" s="66" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C37" s="67"/>
       <c r="D37" s="67"/>
@@ -1874,7 +1873,7 @@
     </row>
     <row r="38" spans="1:6" ht="21" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A38" s="71" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B38" s="7"/>
       <c r="C38" s="7"/>
@@ -1895,16 +1894,16 @@
         <v>21</v>
       </c>
       <c r="B40" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C40" s="53" t="s">
         <v>31</v>
-      </c>
-      <c r="C40" s="53" t="s">
-        <v>32</v>
       </c>
       <c r="D40" s="5" t="s">
         <v>24</v>
       </c>
       <c r="E40" s="53" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F40" s="54" t="s">
         <v>26</v>
@@ -1939,7 +1938,7 @@
     <row r="43" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="80"/>
       <c r="B43" s="81" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C43" s="81"/>
       <c r="D43" s="81"/>
@@ -1957,7 +1956,7 @@
       <c r="B44" s="84"/>
       <c r="C44" s="84"/>
       <c r="D44" s="85" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E44" s="86"/>
       <c r="F44" s="87">
@@ -1972,29 +1971,29 @@
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="90" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B46" s="91"/>
       <c r="E46" s="92" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F46" s="93"/>
     </row>
     <row r="47" spans="1:6" s="70" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A47" s="90" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B47" s="91"/>
       <c r="C47" s="3"/>
       <c r="D47" s="3"/>
       <c r="E47" s="94" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F47" s="95"/>
     </row>
     <row r="48" spans="1:6" s="9" customFormat="1" ht="20.25" x14ac:dyDescent="0.3">
       <c r="A48" s="90" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B48" s="91"/>
       <c r="C48" s="3"/>
@@ -2006,19 +2005,19 @@
       <c r="A49" s="96"/>
       <c r="B49" s="97"/>
       <c r="E49" s="94" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F49" s="95"/>
     </row>
     <row r="50" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B50" s="1"/>
       <c r="C50" s="1"/>
       <c r="D50" s="1"/>
       <c r="E50" s="31" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F50" s="98"/>
     </row>
@@ -2032,7 +2031,7 @@
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B52" s="1"/>
       <c r="C52" s="1"/>
@@ -2050,7 +2049,7 @@
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="101" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B54" s="101"/>
       <c r="C54" s="101"/>
@@ -2068,7 +2067,7 @@
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B56" s="1"/>
       <c r="C56" s="1"/>
@@ -2078,7 +2077,7 @@
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="101" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B57" s="101"/>
       <c r="C57" s="101"/>
@@ -2088,7 +2087,7 @@
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="101" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B58" s="101"/>
       <c r="C58" s="101"/>
@@ -2098,7 +2097,7 @@
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" s="101" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B59" s="101"/>
       <c r="C59" s="101"/>
@@ -2108,7 +2107,7 @@
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="101" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B60" s="101"/>
       <c r="C60" s="101"/>
@@ -2118,7 +2117,7 @@
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="101" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B61" s="101"/>
       <c r="C61" s="101"/>
@@ -2147,7 +2146,7 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="29" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B65" s="29"/>
       <c r="C65" s="29"/>

</xml_diff>